<commit_message>
changes for ros commands
</commit_message>
<xml_diff>
--- a/newui_Greyform/PBU_TERRAHL2.xlsx
+++ b/newui_Greyform/PBU_TERRAHL2.xlsx
@@ -430,6 +430,11 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 0</t>
+        </is>
+      </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Wall Number</t>
@@ -497,7 +502,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="n">
@@ -545,7 +550,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" t="n">
         <v>2</v>
       </c>
       <c r="B3" t="n">
@@ -593,7 +598,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" t="n">
         <v>3</v>
       </c>
       <c r="B4" t="n">
@@ -641,7 +646,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" t="n">
         <v>4</v>
       </c>
       <c r="B5" t="n">
@@ -689,7 +694,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" t="n">
         <v>5</v>
       </c>
       <c r="B6" t="n">
@@ -734,12 +739,12 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
+      <c r="A7" t="n">
         <v>6</v>
       </c>
       <c r="B7" t="n">
@@ -784,12 +789,12 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
+      <c r="A8" t="n">
         <v>7</v>
       </c>
       <c r="B8" t="n">
@@ -834,12 +839,12 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
+      <c r="A9" t="n">
         <v>8</v>
       </c>
       <c r="B9" t="n">
@@ -884,12 +889,12 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
+      <c r="A10" t="n">
         <v>9</v>
       </c>
       <c r="B10" t="n">
@@ -934,12 +939,12 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
+      <c r="A11" t="n">
         <v>10</v>
       </c>
       <c r="B11" t="n">
@@ -984,12 +989,12 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
+      <c r="A12" t="n">
         <v>11</v>
       </c>
       <c r="B12" t="n">
@@ -1034,12 +1039,12 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
+      <c r="A13" t="n">
         <v>12</v>
       </c>
       <c r="B13" t="n">
@@ -1084,12 +1089,12 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
+      <c r="A14" t="n">
         <v>13</v>
       </c>
       <c r="B14" t="n">
@@ -1134,12 +1139,12 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
+      <c r="A15" t="n">
         <v>14</v>
       </c>
       <c r="B15" t="n">
@@ -1184,12 +1189,12 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
+      <c r="A16" t="n">
         <v>15</v>
       </c>
       <c r="B16" t="n">
@@ -1234,12 +1239,12 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
+      <c r="A17" t="n">
         <v>16</v>
       </c>
       <c r="B17" t="n">
@@ -1284,12 +1289,12 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="n">
+      <c r="A18" t="n">
         <v>17</v>
       </c>
       <c r="B18" t="n">
@@ -1334,12 +1339,12 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="n">
+      <c r="A19" t="n">
         <v>18</v>
       </c>
       <c r="B19" t="n">
@@ -1384,12 +1389,12 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="n">
+      <c r="A20" t="n">
         <v>19</v>
       </c>
       <c r="B20" t="n">
@@ -1434,12 +1439,12 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n">
+      <c r="A21" t="n">
         <v>20</v>
       </c>
       <c r="B21" t="n">
@@ -1484,12 +1489,12 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="n">
+      <c r="A22" t="n">
         <v>21</v>
       </c>
       <c r="B22" t="n">
@@ -1534,12 +1539,12 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="n">
+      <c r="A23" t="n">
         <v>22</v>
       </c>
       <c r="B23" t="n">
@@ -1584,12 +1589,12 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="n">
+      <c r="A24" t="n">
         <v>23</v>
       </c>
       <c r="B24" t="n">
@@ -1634,12 +1639,12 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="n">
+      <c r="A25" t="n">
         <v>24</v>
       </c>
       <c r="B25" t="n">
@@ -1684,12 +1689,12 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="n">
+      <c r="A26" t="n">
         <v>25</v>
       </c>
       <c r="B26" t="n">
@@ -1737,7 +1742,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="n">
+      <c r="A27" t="n">
         <v>26</v>
       </c>
       <c r="B27" t="n">
@@ -1785,7 +1790,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="n">
+      <c r="A28" t="n">
         <v>27</v>
       </c>
       <c r="B28" t="n">
@@ -1833,7 +1838,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="n">
+      <c r="A29" t="n">
         <v>28</v>
       </c>
       <c r="B29" t="n">
@@ -1878,12 +1883,12 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="n">
+      <c r="A30" t="n">
         <v>29</v>
       </c>
       <c r="B30" t="n">
@@ -1928,12 +1933,12 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="n">
+      <c r="A31" t="n">
         <v>30</v>
       </c>
       <c r="B31" t="n">
@@ -1978,12 +1983,12 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="n">
+      <c r="A32" t="n">
         <v>31</v>
       </c>
       <c r="B32" t="n">
@@ -2028,12 +2033,12 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="n">
+      <c r="A33" t="n">
         <v>32</v>
       </c>
       <c r="B33" t="n">
@@ -2078,12 +2083,12 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="n">
+      <c r="A34" t="n">
         <v>33</v>
       </c>
       <c r="B34" t="n">
@@ -2128,12 +2133,12 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="n">
+      <c r="A35" t="n">
         <v>34</v>
       </c>
       <c r="B35" t="n">
@@ -2178,12 +2183,12 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1" t="n">
+      <c r="A36" t="n">
         <v>35</v>
       </c>
       <c r="B36" t="n">
@@ -2228,12 +2233,12 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1" t="n">
+      <c r="A37" t="n">
         <v>36</v>
       </c>
       <c r="B37" t="n">
@@ -2278,12 +2283,12 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1" t="n">
+      <c r="A38" t="n">
         <v>37</v>
       </c>
       <c r="B38" t="n">
@@ -2328,12 +2333,12 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1" t="n">
+      <c r="A39" t="n">
         <v>38</v>
       </c>
       <c r="B39" t="n">
@@ -2378,12 +2383,12 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1" t="n">
+      <c r="A40" t="n">
         <v>39</v>
       </c>
       <c r="B40" t="n">
@@ -2428,12 +2433,12 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1" t="n">
+      <c r="A41" t="n">
         <v>40</v>
       </c>
       <c r="B41" t="n">
@@ -2481,7 +2486,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1" t="n">
+      <c r="A42" t="n">
         <v>41</v>
       </c>
       <c r="B42" t="n">
@@ -2529,7 +2534,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1" t="n">
+      <c r="A43" t="n">
         <v>42</v>
       </c>
       <c r="B43" t="n">
@@ -2577,7 +2582,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1" t="n">
+      <c r="A44" t="n">
         <v>43</v>
       </c>
       <c r="B44" t="n">
@@ -2622,12 +2627,12 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1" t="n">
+      <c r="A45" t="n">
         <v>44</v>
       </c>
       <c r="B45" t="n">
@@ -2672,12 +2677,12 @@
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1" t="n">
+      <c r="A46" t="n">
         <v>45</v>
       </c>
       <c r="B46" t="n">
@@ -2722,12 +2727,12 @@
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1" t="n">
+      <c r="A47" t="n">
         <v>46</v>
       </c>
       <c r="B47" t="n">
@@ -2772,12 +2777,12 @@
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1" t="n">
+      <c r="A48" t="n">
         <v>47</v>
       </c>
       <c r="B48" t="n">
@@ -2822,12 +2827,12 @@
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="1" t="n">
+      <c r="A49" t="n">
         <v>48</v>
       </c>
       <c r="B49" t="n">
@@ -2872,12 +2877,12 @@
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="1" t="n">
+      <c r="A50" t="n">
         <v>49</v>
       </c>
       <c r="B50" t="n">
@@ -2922,12 +2927,12 @@
       </c>
       <c r="N50" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="1" t="n">
+      <c r="A51" t="n">
         <v>50</v>
       </c>
       <c r="B51" t="n">
@@ -2972,12 +2977,12 @@
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="1" t="n">
+      <c r="A52" t="n">
         <v>51</v>
       </c>
       <c r="B52" t="n">
@@ -3022,12 +3027,12 @@
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="1" t="n">
+      <c r="A53" t="n">
         <v>52</v>
       </c>
       <c r="B53" t="n">
@@ -3072,12 +3077,12 @@
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="1" t="n">
+      <c r="A54" t="n">
         <v>53</v>
       </c>
       <c r="B54" t="n">
@@ -3122,12 +3127,12 @@
       </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="1" t="n">
+      <c r="A55" t="n">
         <v>54</v>
       </c>
       <c r="B55" t="n">
@@ -3172,12 +3177,12 @@
       </c>
       <c r="N55" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="1" t="n">
+      <c r="A56" t="n">
         <v>55</v>
       </c>
       <c r="B56" t="n">
@@ -3225,7 +3230,7 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="1" t="n">
+      <c r="A57" t="n">
         <v>56</v>
       </c>
       <c r="B57" t="n">
@@ -3273,7 +3278,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="1" t="n">
+      <c r="A58" t="n">
         <v>57</v>
       </c>
       <c r="B58" t="n">
@@ -3321,7 +3326,7 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="1" t="n">
+      <c r="A59" t="n">
         <v>58</v>
       </c>
       <c r="B59" t="n">
@@ -3366,12 +3371,12 @@
       </c>
       <c r="N59" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="1" t="n">
+      <c r="A60" t="n">
         <v>59</v>
       </c>
       <c r="B60" t="n">
@@ -3416,12 +3421,12 @@
       </c>
       <c r="N60" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="1" t="n">
+      <c r="A61" t="n">
         <v>60</v>
       </c>
       <c r="B61" t="n">
@@ -3466,12 +3471,12 @@
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="1" t="n">
+      <c r="A62" t="n">
         <v>61</v>
       </c>
       <c r="B62" t="n">
@@ -3516,12 +3521,12 @@
       </c>
       <c r="N62" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="1" t="n">
+      <c r="A63" t="n">
         <v>62</v>
       </c>
       <c r="B63" t="n">
@@ -3566,12 +3571,12 @@
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="1" t="n">
+      <c r="A64" t="n">
         <v>63</v>
       </c>
       <c r="B64" t="n">
@@ -3616,12 +3621,12 @@
       </c>
       <c r="N64" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="1" t="n">
+      <c r="A65" t="n">
         <v>64</v>
       </c>
       <c r="B65" t="n">
@@ -3666,12 +3671,12 @@
       </c>
       <c r="N65" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="1" t="n">
+      <c r="A66" t="n">
         <v>65</v>
       </c>
       <c r="B66" t="n">
@@ -3716,12 +3721,12 @@
       </c>
       <c r="N66" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="1" t="n">
+      <c r="A67" t="n">
         <v>66</v>
       </c>
       <c r="B67" t="n">
@@ -3769,7 +3774,7 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="1" t="n">
+      <c r="A68" t="n">
         <v>67</v>
       </c>
       <c r="B68" t="n">
@@ -3817,7 +3822,7 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="1" t="n">
+      <c r="A69" t="n">
         <v>68</v>
       </c>
       <c r="B69" t="n">
@@ -3865,7 +3870,7 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="1" t="n">
+      <c r="A70" t="n">
         <v>69</v>
       </c>
       <c r="B70" t="n">
@@ -3910,12 +3915,12 @@
       </c>
       <c r="N70" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="1" t="n">
+      <c r="A71" t="n">
         <v>70</v>
       </c>
       <c r="B71" t="n">
@@ -3960,12 +3965,12 @@
       </c>
       <c r="N71" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="1" t="n">
+      <c r="A72" t="n">
         <v>71</v>
       </c>
       <c r="B72" t="n">
@@ -4010,12 +4015,12 @@
       </c>
       <c r="N72" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="1" t="n">
+      <c r="A73" t="n">
         <v>72</v>
       </c>
       <c r="B73" t="n">
@@ -4063,7 +4068,7 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="1" t="n">
+      <c r="A74" t="n">
         <v>73</v>
       </c>
       <c r="B74" t="n">
@@ -4111,7 +4116,7 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="1" t="n">
+      <c r="A75" t="n">
         <v>74</v>
       </c>
       <c r="B75" t="n">
@@ -4159,7 +4164,7 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="1" t="n">
+      <c r="A76" t="n">
         <v>75</v>
       </c>
       <c r="B76" t="n">
@@ -4204,12 +4209,12 @@
       </c>
       <c r="N76" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="1" t="n">
+      <c r="A77" t="n">
         <v>76</v>
       </c>
       <c r="B77" t="n">
@@ -4254,12 +4259,12 @@
       </c>
       <c r="N77" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="1" t="n">
+      <c r="A78" t="n">
         <v>77</v>
       </c>
       <c r="B78" t="n">
@@ -4304,12 +4309,12 @@
       </c>
       <c r="N78" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="1" t="n">
+      <c r="A79" t="n">
         <v>78</v>
       </c>
       <c r="B79" t="n">
@@ -4354,12 +4359,12 @@
       </c>
       <c r="N79" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="1" t="n">
+      <c r="A80" t="n">
         <v>79</v>
       </c>
       <c r="B80" t="n">
@@ -4404,12 +4409,12 @@
       </c>
       <c r="N80" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="1" t="n">
+      <c r="A81" t="n">
         <v>80</v>
       </c>
       <c r="B81" t="n">
@@ -4454,12 +4459,12 @@
       </c>
       <c r="N81" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="1" t="n">
+      <c r="A82" t="n">
         <v>81</v>
       </c>
       <c r="B82" t="n">
@@ -4504,12 +4509,12 @@
       </c>
       <c r="N82" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="1" t="n">
+      <c r="A83" t="n">
         <v>82</v>
       </c>
       <c r="B83" t="n">
@@ -4554,12 +4559,12 @@
       </c>
       <c r="N83" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="1" t="n">
+      <c r="A84" t="n">
         <v>83</v>
       </c>
       <c r="B84" t="n">
@@ -4604,12 +4609,12 @@
       </c>
       <c r="N84" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="1" t="n">
+      <c r="A85" t="n">
         <v>84</v>
       </c>
       <c r="B85" t="n">
@@ -4654,12 +4659,12 @@
       </c>
       <c r="N85" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="1" t="n">
+      <c r="A86" t="n">
         <v>85</v>
       </c>
       <c r="B86" t="n">
@@ -4704,12 +4709,12 @@
       </c>
       <c r="N86" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="1" t="n">
+      <c r="A87" t="n">
         <v>86</v>
       </c>
       <c r="B87" t="n">
@@ -4754,12 +4759,12 @@
       </c>
       <c r="N87" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="1" t="n">
+      <c r="A88" t="n">
         <v>87</v>
       </c>
       <c r="B88" t="n">
@@ -4804,12 +4809,12 @@
       </c>
       <c r="N88" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="1" t="n">
+      <c r="A89" t="n">
         <v>88</v>
       </c>
       <c r="B89" t="n">
@@ -4854,12 +4859,12 @@
       </c>
       <c r="N89" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="1" t="n">
+      <c r="A90" t="n">
         <v>89</v>
       </c>
       <c r="B90" t="n">
@@ -4904,12 +4909,12 @@
       </c>
       <c r="N90" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="1" t="n">
+      <c r="A91" t="n">
         <v>90</v>
       </c>
       <c r="B91" t="n">
@@ -4954,12 +4959,12 @@
       </c>
       <c r="N91" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="1" t="n">
+      <c r="A92" t="n">
         <v>91</v>
       </c>
       <c r="B92" t="inlineStr">
@@ -5009,7 +5014,7 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="1" t="n">
+      <c r="A93" t="n">
         <v>92</v>
       </c>
       <c r="B93" t="inlineStr">
@@ -5054,12 +5059,12 @@
       </c>
       <c r="N93" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="1" t="n">
+      <c r="A94" t="n">
         <v>93</v>
       </c>
       <c r="B94" t="inlineStr">
@@ -5104,12 +5109,12 @@
       </c>
       <c r="N94" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="1" t="n">
+      <c r="A95" t="n">
         <v>94</v>
       </c>
       <c r="B95" t="inlineStr">
@@ -5154,12 +5159,12 @@
       </c>
       <c r="N95" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="1" t="n">
+      <c r="A96" t="n">
         <v>95</v>
       </c>
       <c r="B96" t="inlineStr">
@@ -5204,12 +5209,12 @@
       </c>
       <c r="N96" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="1" t="n">
+      <c r="A97" t="n">
         <v>96</v>
       </c>
       <c r="B97" t="inlineStr">
@@ -5254,12 +5259,12 @@
       </c>
       <c r="N97" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="1" t="n">
+      <c r="A98" t="n">
         <v>97</v>
       </c>
       <c r="B98" t="inlineStr">
@@ -5304,12 +5309,12 @@
       </c>
       <c r="N98" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="1" t="n">
+      <c r="A99" t="n">
         <v>98</v>
       </c>
       <c r="B99" t="inlineStr">
@@ -5356,12 +5361,12 @@
       </c>
       <c r="N99" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="1" t="n">
+      <c r="A100" t="n">
         <v>99</v>
       </c>
       <c r="B100" t="inlineStr">
@@ -5408,12 +5413,12 @@
       </c>
       <c r="N100" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="1" t="n">
+      <c r="A101" t="n">
         <v>100</v>
       </c>
       <c r="B101" t="inlineStr">
@@ -5460,12 +5465,12 @@
       </c>
       <c r="N101" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="1" t="n">
+      <c r="A102" t="n">
         <v>101</v>
       </c>
       <c r="B102" t="inlineStr">
@@ -5512,12 +5517,12 @@
       </c>
       <c r="N102" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="1" t="n">
+      <c r="A103" t="n">
         <v>102</v>
       </c>
       <c r="B103" t="inlineStr">
@@ -5564,12 +5569,12 @@
       </c>
       <c r="N103" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="1" t="n">
+      <c r="A104" t="n">
         <v>103</v>
       </c>
       <c r="B104" t="inlineStr">
@@ -5616,12 +5621,12 @@
       </c>
       <c r="N104" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="1" t="n">
+      <c r="A105" t="n">
         <v>104</v>
       </c>
       <c r="B105" t="inlineStr">
@@ -5668,12 +5673,12 @@
       </c>
       <c r="N105" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="1" t="n">
+      <c r="A106" t="n">
         <v>105</v>
       </c>
       <c r="B106" t="inlineStr">
@@ -5720,12 +5725,12 @@
       </c>
       <c r="N106" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="1" t="n">
+      <c r="A107" t="n">
         <v>106</v>
       </c>
       <c r="B107" t="inlineStr">
@@ -5772,12 +5777,12 @@
       </c>
       <c r="N107" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="1" t="n">
+      <c r="A108" t="n">
         <v>107</v>
       </c>
       <c r="B108" t="inlineStr">
@@ -5824,12 +5829,12 @@
       </c>
       <c r="N108" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="1" t="n">
+      <c r="A109" t="n">
         <v>108</v>
       </c>
       <c r="B109" t="inlineStr">
@@ -5876,12 +5881,12 @@
       </c>
       <c r="N109" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="1" t="n">
+      <c r="A110" t="n">
         <v>109</v>
       </c>
       <c r="B110" t="inlineStr">
@@ -5928,12 +5933,12 @@
       </c>
       <c r="N110" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="1" t="n">
+      <c r="A111" t="n">
         <v>110</v>
       </c>
       <c r="B111" t="inlineStr">
@@ -5980,12 +5985,12 @@
       </c>
       <c r="N111" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="1" t="n">
+      <c r="A112" t="n">
         <v>111</v>
       </c>
       <c r="B112" t="inlineStr">
@@ -6032,12 +6037,12 @@
       </c>
       <c r="N112" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="1" t="n">
+      <c r="A113" t="n">
         <v>112</v>
       </c>
       <c r="B113" t="inlineStr">
@@ -6084,12 +6089,12 @@
       </c>
       <c r="N113" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="1" t="n">
+      <c r="A114" t="n">
         <v>113</v>
       </c>
       <c r="B114" t="inlineStr">
@@ -6136,12 +6141,12 @@
       </c>
       <c r="N114" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="1" t="n">
+      <c r="A115" t="n">
         <v>114</v>
       </c>
       <c r="B115" t="inlineStr">
@@ -6188,12 +6193,12 @@
       </c>
       <c r="N115" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="1" t="n">
+      <c r="A116" t="n">
         <v>115</v>
       </c>
       <c r="B116" t="inlineStr">
@@ -6240,12 +6245,12 @@
       </c>
       <c r="N116" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="1" t="n">
+      <c r="A117" t="n">
         <v>116</v>
       </c>
       <c r="B117" t="inlineStr">
@@ -6292,12 +6297,12 @@
       </c>
       <c r="N117" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="1" t="n">
+      <c r="A118" t="n">
         <v>117</v>
       </c>
       <c r="B118" t="inlineStr">
@@ -6344,7 +6349,7 @@
       </c>
       <c r="N118" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
@@ -6363,6 +6368,11 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 0</t>
+        </is>
+      </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Wall Number</t>
@@ -6430,7 +6440,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="n">
@@ -6475,12 +6485,12 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" t="n">
         <v>2</v>
       </c>
       <c r="B3" t="n">
@@ -6525,12 +6535,12 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" t="n">
         <v>3</v>
       </c>
       <c r="B4" t="n">
@@ -6575,12 +6585,12 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" t="n">
         <v>4</v>
       </c>
       <c r="B5" t="n">
@@ -6625,12 +6635,12 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" t="n">
         <v>5</v>
       </c>
       <c r="B6" t="n">
@@ -6675,12 +6685,12 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
+      <c r="A7" t="n">
         <v>6</v>
       </c>
       <c r="B7" t="n">
@@ -6725,12 +6735,12 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
+      <c r="A8" t="n">
         <v>7</v>
       </c>
       <c r="B8" t="n">
@@ -6775,12 +6785,12 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
+      <c r="A9" t="n">
         <v>8</v>
       </c>
       <c r="B9" t="n">
@@ -6825,12 +6835,12 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
+      <c r="A10" t="n">
         <v>9</v>
       </c>
       <c r="B10" t="inlineStr">
@@ -6877,12 +6887,12 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
+      <c r="A11" t="n">
         <v>10</v>
       </c>
       <c r="B11" t="inlineStr">
@@ -6929,7 +6939,7 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>done</t>
         </is>
       </c>
     </row>

</xml_diff>